<commit_message>
Reconcile list variables; add List Vars tab to the workbook
list1 = Page: Error (page view + Site Error) AND Form: Error Name (Form
Error Tracking) - a shared/unified error list carried from the source
(parity, flagged for analytics-owner confirm). list2 = Content: Hidden
Tags. list3 unused. Added a List Vars tab to
data-collection-reconciliation.xlsx and issue #10 (list1 shared);
recorded listVars in events-catalog.json _reportSuiteReconciliation.
Report suite List Variables config not captured - noted as the one
remaining screenshot needed for a full names/delimiters reconciliation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L22pJWjoypJEHfB9cqhWZF
</commit_message>
<xml_diff>
--- a/websdk-property/docs/data-collection-reconciliation.xlsx
+++ b/websdk-property/docs/data-collection-reconciliation.xlsx
@@ -12,14 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Elements" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Issues" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List Vars" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Issues" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'eVars'!$A$1:$G$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Props'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Events'!$A$1:$E$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Elements'!$A$1:$D$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Issues'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'List Vars'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Issues'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5556,7 +5558,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>List Var</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Report Suite Name</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Data Element(s)</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Sent By Rule(s)</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Notes / Issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>list1</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>(config not captured — see note)</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Collected</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>Form: Error Name; Page: Error</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>Form Error Tracking; Global Page Load Rule; Site Error</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>SHARED list: carries Form: Error Name + Page: Error from different rules (a unified error list). Parity with the source property — confirm with the analytics owner it is intended, not a collision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>list2</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>(config not captured — see note)</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Collected</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>Content: Hidden Tags</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Global Page Load Rule</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>list3</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>(config not captured)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Defined, old property never sent</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Not populated by this build. Adobe supports list1-3; provide the report suite List Variables config (Admin &gt; Report Suite &gt; Edit Settings &gt; Conversion &gt; List Variables) to reconcile names/delimiters.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5875,32 +6024,62 @@
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
+          <t>list1 shared across error types</t>
+        </is>
+      </c>
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>list1 · Page: Error · Form: Error Name</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>list1 carries Site Error (page views + Site Error rule) AND Form Error Name (Form Error Tracking) — a unified error list. Carried from the source property (parity).</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>Confirm with the analytics owner that list1 is intended as a combined error list. Provide the report suite List Variables config to reconcile names/delimiters and confirm list3 status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
           <t>Empty values omitted</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
       </c>
-      <c r="D11" s="34" t="inlineStr">
+      <c r="D12" s="34" t="inlineStr">
         <is>
           <t>All payloads</t>
         </is>
       </c>
-      <c r="E11" s="34" t="inlineStr">
+      <c r="E12" s="34" t="inlineStr">
         <is>
           <t>The Web SDK build omits empty values, whereas the old XDM elements could emit empty strings. Beacons are cleaner but hit-level QA diffs will show absent-vs-empty differences.</t>
         </is>
       </c>
-      <c r="F11" s="34" t="inlineStr">
+      <c r="F12" s="34" t="inlineStr">
         <is>
           <t>Expected behavior — note for anyone comparing old vs new beacons during QA.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>